<commit_message>
fix： add volume analysis
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_sysbio.xlsx
+++ b/data/proteomics/membrane_size_sysbio.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,664 +443,235 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Glucose_phase(mmol/gDW)</t>
+          <t>prot.1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.2472249023899</v>
+        <v>11.74468831004702</v>
       </c>
       <c r="C2" t="n">
-        <v>12.88753212915063</v>
+        <v>11.96798300720349</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Diauxic_shift(mmol/gDW)</t>
+          <t>prot.2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15.26175688720207</v>
+        <v>11.57464858811228</v>
       </c>
       <c r="C3" t="n">
-        <v>21.25683274981846</v>
+        <v>10.63797793063025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Ethanol_phase(mmol/gDW)</t>
+          <t>prot.3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>19.10013002423777</v>
+        <v>13.30954816470294</v>
       </c>
       <c r="C4" t="n">
-        <v>30.09019901597826</v>
+        <v>11.04891183769896</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>mmol/gDW_carl</t>
+          <t>prot.7</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11.38161699243164</v>
+        <v>7.932605659241445</v>
       </c>
       <c r="C5" t="n">
-        <v>9.943694881111727</v>
+        <v>11.46400124162111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>prot.1</t>
+          <t>prot.8</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12.22072760962364</v>
+        <v>9.177262844617751</v>
       </c>
       <c r="C6" t="n">
-        <v>12.62604490502813</v>
+        <v>11.99145363411174</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>prot.2</t>
+          <t>prot.9</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12.0506878876889</v>
+        <v>11.5562305040926</v>
       </c>
       <c r="C7" t="n">
-        <v>11.29603982845489</v>
+        <v>12.19032884210904</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>prot.3</t>
+          <t>prot.10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13.78558746427956</v>
+        <v>13.03321573353821</v>
       </c>
       <c r="C8" t="n">
-        <v>11.7069737355236</v>
+        <v>18.55529411931943</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>prot.4</t>
+          <t>prot.11</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15.13746210191586</v>
+        <v>11.03668794767441</v>
       </c>
       <c r="C9" t="n">
-        <v>17.39067926677453</v>
+        <v>15.70319113339426</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>prot.5</t>
+          <t>prot.12</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15.67265081220053</v>
+        <v>10.77759926289428</v>
       </c>
       <c r="C10" t="n">
-        <v>17.48655600864473</v>
+        <v>16.79658966470859</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>prot.6</t>
+          <t>prot.13</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13.30069491877897</v>
+        <v>10.98570927108741</v>
       </c>
       <c r="C11" t="n">
-        <v>17.23477189196499</v>
+        <v>18.74889404832998</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>prot.7</t>
+          <t>prot.14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8.408644958818062</v>
+        <v>10.39127525114128</v>
       </c>
       <c r="C12" t="n">
-        <v>12.12206313944575</v>
+        <v>17.95057679292525</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>prot.8</t>
+          <t>prot.15</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9.65330214419437</v>
+        <v>11.36084980929351</v>
       </c>
       <c r="C13" t="n">
-        <v>12.64951553193638</v>
+        <v>19.19462775344603</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>prot.9</t>
+          <t>prot.16</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12.03226980366921</v>
+        <v>13.15461716256718</v>
       </c>
       <c r="C14" t="n">
-        <v>12.84839073993368</v>
+        <v>25.36960725565431</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>prot.10</t>
+          <t>prot.17</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13.50925503311483</v>
+        <v>13.52386684921094</v>
       </c>
       <c r="C15" t="n">
-        <v>19.21335601714406</v>
+        <v>24.43408699235508</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>prot.11</t>
+          <t>prot.18</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11.51272724725103</v>
+        <v>11.77836445965474</v>
       </c>
       <c r="C16" t="n">
-        <v>16.3612530312189</v>
+        <v>21.8208432163772</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>prot.12</t>
+          <t>prot.19</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>11.2536385624709</v>
+        <v>13.25511093809547</v>
       </c>
       <c r="C17" t="n">
-        <v>17.45465156253322</v>
+        <v>23.67331946297611</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>prot.13</t>
+          <t>prot.20</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11.46174857066403</v>
+        <v>14.23732749813225</v>
       </c>
       <c r="C18" t="n">
-        <v>19.40695594615461</v>
+        <v>26.11959170561098</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>prot.14</t>
+          <t>prot.21</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10.8673145507179</v>
+        <v>14.49364331332636</v>
       </c>
       <c r="C19" t="n">
-        <v>18.60863869074987</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>prot.15</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>11.83688910887013</v>
-      </c>
-      <c r="C20" t="n">
-        <v>19.85268965127065</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>prot.16</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>13.6306564621438</v>
-      </c>
-      <c r="C21" t="n">
-        <v>26.02766915347893</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>prot.17</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>13.99990614878756</v>
-      </c>
-      <c r="C22" t="n">
-        <v>25.0921488901797</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>prot.18</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>12.25440375923136</v>
-      </c>
-      <c r="C23" t="n">
-        <v>22.47890511420184</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>prot.19</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>13.73115023767209</v>
-      </c>
-      <c r="C24" t="n">
-        <v>24.33138136080074</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>prot.20</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>14.71336679770886</v>
-      </c>
-      <c r="C25" t="n">
-        <v>26.77765360343562</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>prot.21</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>14.96968261290298</v>
-      </c>
-      <c r="C26" t="n">
-        <v>29.24272179077044</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>prot.22</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>16.43182273746284</v>
-      </c>
-      <c r="C27" t="n">
-        <v>25.76166864582199</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>prot.23</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>20.22592472513374</v>
-      </c>
-      <c r="C28" t="n">
-        <v>28.78827457416135</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>prot.24</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>20.31313093132106</v>
-      </c>
-      <c r="C29" t="n">
-        <v>29.80527444304868</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>prot.25</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>17.79580945554654</v>
-      </c>
-      <c r="C30" t="n">
-        <v>29.75277730645366</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>prot.26</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>11.20315226519365</v>
-      </c>
-      <c r="C31" t="n">
-        <v>16.06992224208038</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>prot.27</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>13.94405103620363</v>
-      </c>
-      <c r="C32" t="n">
-        <v>19.23355353268291</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>prot.28</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>10.98998534121922</v>
-      </c>
-      <c r="C33" t="n">
-        <v>13.06327284794153</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>prot.29</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>17.24826653444831</v>
-      </c>
-      <c r="C34" t="n">
-        <v>23.66005049958389</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>prot.30</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>15.95282814595184</v>
-      </c>
-      <c r="C35" t="n">
-        <v>23.69858741990602</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>prot.31</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>17.77759384165887</v>
-      </c>
-      <c r="C36" t="n">
-        <v>24.70821856060923</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>prot.32</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>20.88439804501617</v>
-      </c>
-      <c r="C37" t="n">
-        <v>30.39595812839542</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>prot.33</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>18.89020368374504</v>
-      </c>
-      <c r="C38" t="n">
-        <v>26.73727553132137</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
-        <is>
-          <t>prot.34</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>19.07770195426369</v>
-      </c>
-      <c r="C39" t="n">
-        <v>26.70195105583313</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>prot.35</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>18.05874825617794</v>
-      </c>
-      <c r="C40" t="n">
-        <v>25.39576934468794</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>prot.36</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>18.10451954340165</v>
-      </c>
-      <c r="C41" t="n">
-        <v>28.57277206658785</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>prot.37</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>11.94245866775519</v>
-      </c>
-      <c r="C42" t="n">
-        <v>20.66586355643068</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>prot.38</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>15.2736117540319</v>
-      </c>
-      <c r="C43" t="n">
-        <v>24.98233070660377</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>prot.39</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>12.16771568972033</v>
-      </c>
-      <c r="C44" t="n">
-        <v>18.22008339599203</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t>prot.40</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>20.60964259659599</v>
-      </c>
-      <c r="C45" t="n">
-        <v>26.02321417818069</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>prot.41</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>19.59827927998146</v>
-      </c>
-      <c r="C46" t="n">
-        <v>28.39873994289943</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>prot.42</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>18.13617499884792</v>
-      </c>
-      <c r="C47" t="n">
-        <v>25.54754171195981</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>mmol/gDW_Tyler_D0.1</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>21.77320723029894</v>
-      </c>
-      <c r="C48" t="n">
-        <v>14.05201052691336</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>Min_ave_aerobic(mmol/gDW)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>15.41778226967429</v>
-      </c>
-      <c r="C49" t="n">
-        <v>10.49044278437261</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>Rich_ave_aerobic(mmol/gDW)</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>16.7214032017335</v>
-      </c>
-      <c r="C50" t="n">
-        <v>11.02898813476818</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>Min_ave_anaerobic(mmol/gDW)</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>12.61055576328672</v>
-      </c>
-      <c r="C51" t="n">
-        <v>6.331961487387513</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>Rich_ave_anaerobic(mmol/gDW)</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>12.90923513925826</v>
-      </c>
-      <c r="C52" t="n">
-        <v>5.755672186621559</v>
+        <v>28.58465989294582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add more data based on yeast cell size data
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_sysbio.xlsx
+++ b/data/proteomics/membrane_size_sysbio.xlsx
@@ -447,10 +447,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.74468831004702</v>
+        <v>8.834259072602098</v>
       </c>
       <c r="C2" t="n">
-        <v>11.96798300720349</v>
+        <v>9.002219528609343</v>
       </c>
     </row>
     <row r="3">
@@ -460,10 +460,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11.57464858811228</v>
+        <v>8.706356576039491</v>
       </c>
       <c r="C3" t="n">
-        <v>10.63797793063025</v>
+        <v>8.001800521808399</v>
       </c>
     </row>
     <row r="4">
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13.30954816470294</v>
+        <v>10.01133393430948</v>
       </c>
       <c r="C4" t="n">
-        <v>11.04891183769896</v>
+        <v>8.310901666166227</v>
       </c>
     </row>
     <row r="5">
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.932605659241445</v>
+        <v>6.530599188264407</v>
       </c>
       <c r="C5" t="n">
-        <v>11.46400124162111</v>
+        <v>9.437856918498603</v>
       </c>
     </row>
     <row r="6">
@@ -499,10 +499,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.177262844617751</v>
+        <v>7.55527601623914</v>
       </c>
       <c r="C6" t="n">
-        <v>11.99145363411174</v>
+        <v>9.872087524962005</v>
       </c>
     </row>
     <row r="7">
@@ -512,10 +512,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11.5562305040926</v>
+        <v>9.513785607318365</v>
       </c>
       <c r="C7" t="n">
-        <v>12.19032884210904</v>
+        <v>10.03581358518788</v>
       </c>
     </row>
     <row r="8">
@@ -525,10 +525,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13.03321573353821</v>
+        <v>11.28547886339388</v>
       </c>
       <c r="C8" t="n">
-        <v>18.55529411931943</v>
+        <v>16.06705389282984</v>
       </c>
     </row>
     <row r="9">
@@ -538,10 +538,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11.03668794767441</v>
+        <v>9.556682794319094</v>
       </c>
       <c r="C9" t="n">
-        <v>15.70319113339426</v>
+        <v>13.5974141184299</v>
       </c>
     </row>
     <row r="10">
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.77759926289428</v>
+        <v>9.33233755707219</v>
       </c>
       <c r="C10" t="n">
-        <v>16.79658966470859</v>
+        <v>14.54418936305817</v>
       </c>
     </row>
     <row r="11">
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10.98570927108741</v>
+        <v>10.29327721599667</v>
       </c>
       <c r="C11" t="n">
-        <v>18.74889404832998</v>
+        <v>17.56714647826358</v>
       </c>
     </row>
     <row r="12">
@@ -577,10 +577,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10.39127525114128</v>
+        <v>9.736310523820679</v>
       </c>
       <c r="C12" t="n">
-        <v>17.95057679292525</v>
+        <v>16.81914736292005</v>
       </c>
     </row>
     <row r="13">
@@ -590,10 +590,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11.36084980929351</v>
+        <v>10.64477255047418</v>
       </c>
       <c r="C13" t="n">
-        <v>19.19462775344603</v>
+        <v>17.98478547434986</v>
       </c>
     </row>
     <row r="14">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13.15461716256718</v>
+        <v>14.5691849331249</v>
       </c>
       <c r="C14" t="n">
-        <v>25.36960725565431</v>
+        <v>28.09770099886684</v>
       </c>
     </row>
     <row r="15">
@@ -616,10 +616,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13.52386684921094</v>
+        <v>14.97814149223479</v>
       </c>
       <c r="C15" t="n">
-        <v>24.43408699235508</v>
+        <v>27.061580558701</v>
       </c>
     </row>
     <row r="16">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11.77836445965474</v>
+        <v>13.04493835903978</v>
       </c>
       <c r="C16" t="n">
-        <v>21.8208432163772</v>
+        <v>24.16732439168008</v>
       </c>
     </row>
     <row r="17">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13.25511093809547</v>
+        <v>15.62250490095466</v>
       </c>
       <c r="C17" t="n">
-        <v>23.67331946297611</v>
+        <v>27.90142995101545</v>
       </c>
     </row>
     <row r="18">
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>14.23732749813225</v>
+        <v>16.78014764680844</v>
       </c>
       <c r="C18" t="n">
-        <v>26.11959170561098</v>
+        <v>30.78461216488866</v>
       </c>
     </row>
     <row r="19">
@@ -668,10 +668,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14.49364331332636</v>
+        <v>17.08224206893463</v>
       </c>
       <c r="C19" t="n">
-        <v>28.58465989294582</v>
+        <v>33.68994732335536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add more simulation
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_sysbio.xlsx
+++ b/data/proteomics/membrane_size_sysbio.xlsx
@@ -447,10 +447,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8.834259072602098</v>
+        <v>8.834259072602096</v>
       </c>
       <c r="C2" t="n">
-        <v>9.002219528609343</v>
+        <v>9.002219528609345</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8.706356576039491</v>
+        <v>8.706356576039489</v>
       </c>
       <c r="C3" t="n">
         <v>8.001800521808399</v>
@@ -476,7 +476,7 @@
         <v>10.01133393430948</v>
       </c>
       <c r="C4" t="n">
-        <v>8.310901666166227</v>
+        <v>8.310901666166226</v>
       </c>
     </row>
     <row r="5">
@@ -499,10 +499,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.55527601623914</v>
+        <v>7.555276016239143</v>
       </c>
       <c r="C6" t="n">
-        <v>9.872087524962005</v>
+        <v>9.872087524962</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9.513785607318365</v>
+        <v>9.51378560731837</v>
       </c>
       <c r="C7" t="n">
         <v>10.03581358518788</v>
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9.33233755707219</v>
+        <v>9.332337557072192</v>
       </c>
       <c r="C10" t="n">
-        <v>14.54418936305817</v>
+        <v>14.54418936305818</v>
       </c>
     </row>
     <row r="11">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.736310523820679</v>
+        <v>9.736310523820672</v>
       </c>
       <c r="C12" t="n">
         <v>16.81914736292005</v>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>10.64477255047418</v>
+        <v>10.64477255047419</v>
       </c>
       <c r="C13" t="n">
         <v>17.98478547434986</v>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15.62250490095466</v>
+        <v>15.62250490095467</v>
       </c>
       <c r="C17" t="n">
         <v>27.90142995101545</v>
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>16.78014764680844</v>
+        <v>16.78014764680845</v>
       </c>
       <c r="C18" t="n">
         <v>30.78461216488866</v>
@@ -668,10 +668,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>17.08224206893463</v>
+        <v>17.08224206893462</v>
       </c>
       <c r="C19" t="n">
-        <v>33.68994732335536</v>
+        <v>33.68994732335538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>